<commit_message>
RESHIPPED (task446): 10/10 repair, CRM-07 5.2 files the estimand only and the data forces the forecasting basis; caseload 133 unchanged
The client returned task446 on the rule-application rule: 5.2 filed the model, the
fitting window and the leave-one-cohort-out selection. 5.2 now files only what is
forecast, 5.3 the band split as a reporting convention; every basis that validates
out of sample files 133, the hit-rate route files 73. prompt.txt replaces prompt.md;
pairing retagged to Forecasting (credit-scoring-pd-modeling); design note brought to
the current precut format. Every graded figure unchanged. Gates: 9,162 checks,
byte-identical rebuilds, precut 49/0, figures_check, leak.py REVIEW only, heart WARN;
leak reader clean; judge DETERMINISTIC, APPROVE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es2YJxT597uNAuNJZNdYR4
</commit_message>
<xml_diff>
--- a/task446/golden/watchlist_inflow_2027.xlsx
+++ b/task446/golden/watchlist_inflow_2027.xlsx
@@ -736,7 +736,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>1  A group's chance of reaching the watch list depends only on its flag at 30 September 2026 (CRM-07 s5.2): 63.0% if flagged AMBER or RED, 3.9% if not, on the basis the s5.2 test selects from the 2022 to 2025 cohorts; see Cohorts.</t>
+          <t>1  A group's chance of reaching the watch list by its flag at 30 September 2026: 63.0% if flagged AMBER or RED, 3.9% if not. Set from the screen's capture and false-alarm rates over the 2022 to 2025 cohorts taken together (CRM-07 s4.3), which hold from year to year, with this year's arrival share backed out of the September flagged share; the hit and miss rates move with each year's arrivals. See Cohorts.</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>5  Computed unrounded. Caseload to the nearest whole group, band figures to one decimal (s5.3); totals rounded from the unrounded sums.</t>
+          <t>5  Computed unrounded. Caseload to the nearest whole group; band arrivals and exposure split by flag status and band figures to one decimal (s5.3); totals rounded from the unrounded sums.</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Choice of basis (CRM-07 s5.2): each closed cohort predicted from the other three taken together</t>
+          <t>Back-test of the forecasting bases: each closed cohort predicted from the other three taken together</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>Monitored book at 30 September 2026 only, no new groups (s5.1). One probability for flagged groups and one for the rest, on the basis with the smallest largest miss when each closed cohort is predicted from the other three taken together (s5.2).</t>
+          <t>Monitored book at 30 September 2026 only, no new groups (s5.1, s5.2). One probability for flagged groups and one for the rest, from the capture and false-alarm rates (s4.3) with this year's arrival share backed out of the flagged share: the basis whose largest miss is smallest when each closed cohort is predicted from the other three taken together (see Cohorts).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PAUSED (task446): stage 4 in flight, two scored readers and the judge thread on the cut pack
Architecture 3's stage 3 gates are green (9329 generator assertions, figures_check,
precut, voice-check, leak.py REVIEW with no LEAK, producer metadata clean). The forum
and forcing event were redrawn in the pack after heart found them banned against
task486 v2: CRM-07 5.1 and 5.2 now make the forecast part of the monitoring year-end
close, from which the chief risk officer's leadership team sets the headcount, and a
Credit Risk Monitoring close timetable replaces the committee agenda. No figure moved.
The write-up drops the rival figures from block 1 and the back-test component, and
states the back-test miss as a level, not a bound. The goldens' footer overlap and rate
rounding are fixed. figures.json is keyed so the readers can be scored.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016XvnoparzX994L4tvvsE27
</commit_message>
<xml_diff>
--- a/task446/golden/watchlist_inflow_2027.xlsx
+++ b/task446/golden/watchlist_inflow_2027.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -137,12 +137,6 @@
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -521,8 +515,8 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -543,7 +537,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Executive Risk Committee, 4 November 2026, item 3.1</t>
+          <t>Year-end close pack for the Chief Risk Officer's leadership team, 4 November 2026</t>
         </is>
       </c>
     </row>
@@ -554,7 +548,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>133</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6">
@@ -584,14 +578,14 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Expected arrivals,
-flagged in September</t>
+          <t>Flagged in
+September</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Expected arrivals,
-not flagged</t>
+          <t>Expected
+arrivals</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -611,16 +605,16 @@
         <v>201</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>475.8</v>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>21.4</v>
+        <v>499.9</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>34</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>6.5</v>
+        <v>16.2</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>69.59999999999999</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="10">
@@ -630,19 +624,19 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3016.2</v>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>34</v>
+        <v>3112</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>54</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>9.800000000000001</v>
+        <v>25.8</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>411.5</v>
+        <v>257.1</v>
       </c>
     </row>
     <row r="11">
@@ -652,19 +646,19 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>7153.8</v>
-      </c>
-      <c r="D11" s="10" t="n">
-        <v>29.6</v>
+        <v>6936.6</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>7.9</v>
+        <v>21.9</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1108.6</v>
+        <v>596.8</v>
       </c>
     </row>
     <row r="12">
@@ -677,16 +671,16 @@
         <v>120</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>8213.799999999999</v>
-      </c>
-      <c r="D12" s="10" t="n">
-        <v>12.6</v>
+        <v>8402.700000000001</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>20</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>3.9</v>
+        <v>9</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>1121.5</v>
+        <v>576.3</v>
       </c>
     </row>
     <row r="13">
@@ -696,19 +690,19 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>6640.9</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>6.3</v>
+        <v>6712.2</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>11</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>1</v>
+        <v>5.1</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>1283.4</v>
+        <v>826.8</v>
       </c>
     </row>
     <row r="14">
@@ -721,29 +715,29 @@
         <v>913</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>25500.5</v>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>103.9</v>
+        <v>25663.4</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>165</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>29.1</v>
+        <v>78</v>
       </c>
       <c r="F14" s="13" t="n">
-        <v>3994.6</v>
+        <v>2295.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>1  A group's chance of reaching the watch list by its flag at 30 September 2026: 63.0% if flagged AMBER or RED, 3.9% if not. Set from the screen's capture and false-alarm rates over the 2022 to 2025 cohorts taken together (CRM-07 s4.3), which hold from year to year, with this year's arrival share backed out of the September flagged share; the hit and miss rates move with each year's arrivals. See Cohorts.</t>
+          <t>1  Chance of reaching the watch list within the year, by the September flag: 50.0% where the flag was raised on a customer we lend to, 6.25% where it was raised only on a parent or sister company we do not lend to, 1.62% where the group was not flagged. Set from the 2022 to 2025 cohorts taken together; see Cohorts.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>2  Committed exposure per CRM-07 s6.1: every facility on which a member is an obligor, once per group (a joint facility counts in each of its groups), at its limit as it stood at the end of 30 September UK time (23:00 UTC in the limit history), in sterling at Group Treasury closing rates.</t>
+          <t>2  Committed exposure per CRM-07 s6.1: every facility on which a member is an obligor, once per group (a joint facility counts in each of its groups, and so does the facility of a company booked to one group and consolidated into another under s2.2), at its limit as it stood at the end of 30 September UK time (23:00 UTC in the limit history), in sterling at Group Treasury closing rates.</t>
         </is>
       </c>
     </row>
@@ -764,7 +758,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>5  Computed unrounded. Caseload to the nearest whole group; band arrivals and exposure split by flag status and band figures to one decimal (s5.3); totals rounded from the unrounded sums.</t>
+          <t>5  Computed unrounded. Caseload to the nearest whole group, band arrivals and exposure to one decimal (s5.3); totals rounded from the unrounded sums.</t>
         </is>
       </c>
     </row>
@@ -780,24 +774,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Early-warning performance on the closed cohorts (CRM-07 s4.3)</t>
+          <t>Closed cohorts, by where the September flag was raised</t>
         </is>
       </c>
     </row>
@@ -815,41 +809,41 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Flagged</t>
+          <t>Flagged on a
+customer</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Reached the
-watch list</t>
+          <t>Reached</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Flagged and
-reached</t>
+          <t>Flagged only on
+a non-customer</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Hit rate</t>
+          <t>Reached</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Capture rate</t>
+          <t>Not
+flagged</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>False-alarm
-rate</t>
+          <t>Reached</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>Share of book
-reaching</t>
+          <t>Reached,
+all groups</t>
         </is>
       </c>
     </row>
@@ -861,25 +855,25 @@
         <v>846</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>119</v>
+        <v>58</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>58</v>
-      </c>
-      <c r="F4" s="17" t="n">
-        <v>0.4873949579831933</v>
-      </c>
-      <c r="G4" s="17" t="n">
-        <v>0.7733333333333333</v>
-      </c>
-      <c r="H4" s="18" t="n">
-        <v>0.07911802853437094</v>
-      </c>
-      <c r="I4" s="17" t="n">
-        <v>0.08865248226950355</v>
+        <v>62</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>726</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="5">
@@ -890,25 +884,25 @@
         <v>871</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>32</v>
-      </c>
-      <c r="F5" s="17" t="n">
-        <v>0.3265306122448979</v>
-      </c>
-      <c r="G5" s="17" t="n">
-        <v>0.7441860465116279</v>
-      </c>
-      <c r="H5" s="18" t="n">
-        <v>0.07971014492753623</v>
-      </c>
-      <c r="I5" s="17" t="n">
-        <v>0.04936854190585534</v>
+        <v>28</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>781</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -919,25 +913,25 @@
         <v>889</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>95</v>
+        <v>58</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>28</v>
-      </c>
-      <c r="F6" s="17" t="n">
-        <v>0.2947368421052631</v>
-      </c>
-      <c r="G6" s="17" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="H6" s="18" t="n">
-        <v>0.07854630715123095</v>
-      </c>
-      <c r="I6" s="17" t="n">
-        <v>0.04049493813273341</v>
+        <v>40</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>791</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -948,25 +942,25 @@
         <v>902</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>39</v>
-      </c>
-      <c r="F7" s="17" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="G7" s="17" t="n">
-        <v>0.8297872340425532</v>
-      </c>
-      <c r="H7" s="18" t="n">
-        <v>0.07602339181286549</v>
-      </c>
-      <c r="I7" s="17" t="n">
-        <v>0.05210643015521065</v>
+        <v>46</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>794</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -979,528 +973,243 @@
         <v>3508</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>416</v>
+        <v>240</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>201</v>
+        <v>120</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>157</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>0.3774038461538461</v>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>0.7810945273631841</v>
-      </c>
-      <c r="H8" s="20" t="n">
-        <v>0.07831871787118234</v>
-      </c>
-      <c r="I8" s="19" t="n">
-        <v>0.0572976054732041</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Back-test of the forecasting bases: each closed cohort predicted from the other three taken together</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+        <v>176</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>3092</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Share reaching the list</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="H9" s="18" t="n">
+        <v>0.01617076326002587</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>0.0515963511972634</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Each closed cohort forecast from the other three taken together (forecast less actual arrivals, as a share of actual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Miss
-2022</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Miss
-2023</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Miss
-2024</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Miss
-2025</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Largest
 miss</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>2026 book,
 expected</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>Capture and false-alarm rates, share reaching backed out of the flagged share</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="n">
-        <v>-0.002354189884837821</v>
-      </c>
-      <c r="C12" s="22" t="n">
-        <v>-0.01571755433086564</v>
-      </c>
-      <c r="D12" s="22" t="n">
-        <v>0.004586044944293599</v>
-      </c>
-      <c r="E12" s="22" t="n">
-        <v>0.01053415358576126</v>
-      </c>
-      <c r="F12" s="23" t="n">
-        <v>0.01571755433086564</v>
-      </c>
-      <c r="G12" s="24" t="n">
-        <v>133.036751295115</v>
-      </c>
-    </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Share reaching on flagged share, straight line</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n">
-        <v>-0.005129616299269668</v>
-      </c>
-      <c r="C13" s="25" t="n">
-        <v>-0.02001418913908593</v>
-      </c>
-      <c r="D13" s="25" t="n">
-        <v>0.00776767249510546</v>
-      </c>
-      <c r="E13" s="25" t="n">
-        <v>0.01396602549297632</v>
+          <t>One rate for flagged groups, one for the rest</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>0.1441883134190827</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>-0.1120188942542955</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0.0204796777408911</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>-0.03225772269505944</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>0.02001418913908593</v>
+        <v>0.1441883134190827</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>132.8313695619687</v>
+        <v>64.05486553388397</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Share reaching on flagged share, straight line weighted by book</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="n">
-        <v>-0.005554532443961979</v>
-      </c>
-      <c r="C14" s="25" t="n">
-        <v>-0.02004885773708553</v>
-      </c>
-      <c r="D14" s="25" t="n">
-        <v>0.007461624292518287</v>
-      </c>
-      <c r="E14" s="25" t="n">
-        <v>0.01390799109854979</v>
+          <t>A rate by where the flag was raised, one for the rest</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>-0.01157693708301</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>0.0118754833382968</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>0.0391979356249339</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>-0.03616916705594198</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>0.02004885773708553</v>
+        <v>0.0391979356249339</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>132.8339886746333</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Arrivals on flagged groups and book size</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="n">
-        <v>-0.005971624392815844</v>
-      </c>
-      <c r="C15" s="25" t="n">
-        <v>-0.02008377192752864</v>
-      </c>
-      <c r="D15" s="25" t="n">
-        <v>0.007155600104049142</v>
-      </c>
-      <c r="E15" s="25" t="n">
-        <v>0.01385067933119921</v>
-      </c>
-      <c r="F15" s="17" t="n">
-        <v>0.02008377192752864</v>
-      </c>
-      <c r="G15" s="10" t="n">
-        <v>132.836143410683</v>
+        <v>77.97073091849936</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Capture and false-alarm rates, mean of the cohorts' rates</t>
-        </is>
-      </c>
-      <c r="B16" s="25" t="n">
-        <v>-6.982552439638301e-05</v>
-      </c>
-      <c r="C16" s="25" t="n">
-        <v>-0.02027581569971992</v>
-      </c>
-      <c r="D16" s="25" t="n">
-        <v>0.002216703587756497</v>
-      </c>
-      <c r="E16" s="25" t="n">
-        <v>0.01205359957462626</v>
-      </c>
-      <c r="F16" s="17" t="n">
-        <v>0.02027581569971992</v>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>132.9692125764468</v>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Book at 30 September 2026</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hit and miss rates, each trended on flagged share</t>
-        </is>
-      </c>
-      <c r="B17" s="25" t="n">
-        <v>0.07972716809432878</v>
-      </c>
-      <c r="C17" s="25" t="n">
-        <v>-0.02850416575429371</v>
-      </c>
-      <c r="D17" s="25" t="n">
-        <v>0.03410379148627385</v>
-      </c>
-      <c r="E17" s="25" t="n">
-        <v>-0.001600822274049118</v>
-      </c>
-      <c r="F17" s="17" t="n">
-        <v>0.07972716809432878</v>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>146.7205801419634</v>
+          <t>Groups monitored</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>913</v>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>active on the group register and not on the watch list (s4.1)</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hit and miss rates of the latest cohort</t>
-        </is>
-      </c>
-      <c r="B18" s="25" t="n">
-        <v>-0.3078237259816208</v>
-      </c>
-      <c r="C18" s="25" t="n">
-        <v>0.03486914961823162</v>
-      </c>
-      <c r="D18" s="25" t="n">
-        <v>0.2106916597048176</v>
-      </c>
-      <c r="E18" s="25" t="n">
-        <v>-0.176746088384045</v>
-      </c>
-      <c r="F18" s="17" t="n">
-        <v>0.3078237259816208</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>69.37374686716792</v>
+          <t>Flagged AMBER or RED</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>September 2026 publication, any member (s3.2)</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Arrivals per flagged group, none from the rest</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="n">
-        <v>-0.3268686868686869</v>
-      </c>
-      <c r="C19" s="25" t="n">
-        <v>0.1323679976597922</v>
-      </c>
-      <c r="D19" s="25" t="n">
-        <v>0.3564382139148492</v>
-      </c>
-      <c r="E19" s="25" t="n">
-        <v>0.09219858156028371</v>
-      </c>
-      <c r="F19" s="17" t="n">
-        <v>0.3564382139148492</v>
-      </c>
-      <c r="G19" s="10" t="n">
-        <v>79.72355769230769</v>
+          <t xml:space="preserve">  raised on a customer</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>127</v>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>50.0% expected to reach the list</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hit and miss rates, mean of the cohorts' rates</t>
-        </is>
-      </c>
-      <c r="B20" s="25" t="n">
-        <v>-0.3621582571111575</v>
-      </c>
-      <c r="C20" s="25" t="n">
-        <v>0.1396306690736682</v>
-      </c>
-      <c r="D20" s="25" t="n">
-        <v>0.396049788363716</v>
-      </c>
-      <c r="E20" s="25" t="n">
-        <v>0.08763969882439193</v>
-      </c>
-      <c r="F20" s="17" t="n">
-        <v>0.396049788363716</v>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>71.99371779677551</v>
+          <t xml:space="preserve">  raised only on a non-customer</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>6.25% expected to reach the list</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hit and miss rates</t>
-        </is>
-      </c>
-      <c r="B21" s="25" t="n">
-        <v>-0.3604472633309842</v>
-      </c>
-      <c r="C21" s="25" t="n">
-        <v>0.1516747111306129</v>
-      </c>
-      <c r="D21" s="25" t="n">
-        <v>0.4060058997530023</v>
-      </c>
-      <c r="E21" s="25" t="n">
-        <v>0.103328448558373</v>
-      </c>
-      <c r="F21" s="17" t="n">
-        <v>0.4060058997530023</v>
-      </c>
-      <c r="G21" s="10" t="n">
-        <v>72.91587782366405</v>
+          <t>Not flagged</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>748</v>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>1.62% expected to reach the list</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>One share for every group</t>
-        </is>
-      </c>
-      <c r="B22" s="25" t="n">
-        <v>-0.4660856498873028</v>
-      </c>
-      <c r="C22" s="25" t="n">
-        <v>0.2136589323667664</v>
-      </c>
-      <c r="D22" s="25" t="n">
-        <v>0.5557782868779431</v>
-      </c>
-      <c r="E22" s="25" t="n">
-        <v>0.1341095018043468</v>
-      </c>
-      <c r="F22" s="17" t="n">
-        <v>0.5557782868779431</v>
-      </c>
-      <c r="G22" s="10" t="n">
-        <v>52.31271379703535</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Hit and miss rates of the most stressed cohort</t>
-        </is>
-      </c>
-      <c r="B23" s="25" t="n">
-        <v>-0.3078237259816208</v>
-      </c>
-      <c r="C23" s="25" t="n">
-        <v>0.5311711454038766</v>
-      </c>
-      <c r="D23" s="25" t="n">
-        <v>0.801923153488814</v>
-      </c>
-      <c r="E23" s="25" t="n">
-        <v>0.4755175153850939</v>
-      </c>
-      <c r="F23" s="17" t="n">
-        <v>0.801923153488814</v>
-      </c>
-      <c r="G23" s="10" t="n">
-        <v>97.91122721440708</v>
+          <t>Expected arrivals</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>77.97073091849936</v>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>65.9 from flagged groups, 12.1 from the rest; caseload 78</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Every flagged group reaches, the rest at the miss rate</t>
-        </is>
-      </c>
-      <c r="B24" s="25" t="n">
-        <v>0.6973305144467934</v>
-      </c>
-      <c r="C24" s="25" t="n">
-        <v>1.534883720930233</v>
-      </c>
-      <c r="D24" s="25" t="n">
-        <v>1.984406730490281</v>
-      </c>
-      <c r="E24" s="25" t="n">
-        <v>1.479214973381068</v>
-      </c>
-      <c r="F24" s="17" t="n">
-        <v>1.984406730490281</v>
-      </c>
-      <c r="G24" s="10" t="n">
-        <v>175.6442432082794</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>Miss: predicted less actual arrivals, as a share of actual arrivals. Basis used: the smallest largest miss.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Book at 30 September 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Groups monitored</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="n">
-        <v>913</v>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>active on the group register and not on the watch list (s4.1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Flagged AMBER or RED</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="C29" s="1" t="inlineStr">
-        <is>
-          <t>September 2026 publication, any member (s3.2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Flagged share</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="n">
-        <v>0.1807228915662651</v>
-      </c>
-      <c r="C30" s="1" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Share of book expected to reach the list</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="n">
-        <v>0.1457138568402135</v>
-      </c>
-      <c r="C31" s="1" t="inlineStr">
-        <is>
-          <t>(flagged share less false-alarm rate) / (capture rate less false-alarm rate)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Probability of reaching, flagged</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="n">
-        <v>0.6297835053017654</v>
-      </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>capture rate x expected share / flagged share</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Probability of reaching, not flagged</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="n">
-        <v>0.03893378732663592</v>
-      </c>
-      <c r="C33" s="1" t="inlineStr">
-        <is>
-          <t>(1 - capture rate) x expected share / (1 - flagged share)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Expected arrivals</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n">
-        <v>133.036751295115</v>
-      </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>103.9 flagged + 29.1 not flagged; caseload 133</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
-        <is>
-          <t>The hit rate has moved from 29.5% to 48.7% with the share of each cohort that reached the list (4.0% to 8.9%); capture (74.4% to 83.0%) and false-alarm (7.60% to 7.97%) rates have held.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
-        <is>
-          <t>This year 18.1% of the book is flagged, against 10.7% to 14.1% in the closed cohorts.</t>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Customers raised 48% to 69% of the flags in the closed cohorts and 77% of this September's.</t>
         </is>
       </c>
     </row>
@@ -1531,108 +1240,108 @@
       <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>As at</t>
         </is>
       </c>
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Monitored book, flags and committed exposure at 30 September 2026. Forecast window 1 October 2026 to 30 September 2027.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="26" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Obligor groups</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
-        <is>
-          <t>Group register customers plus GLEIF accounting-consolidation members in force at each date (CRM-07 s2.2). Engine signals keyed by LEI or Companies House number.</t>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>The ultimate parent, the customers the credit system books to the group and the GLEIF accounting-consolidation members in force at each date (CRM-07 s2.2). Engine signals keyed by LEI or Companies House number.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
-        <is>
-          <t>Any member AMBER or RED in the engine's month-end publication for the date (s3.2).</t>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Any member AMBER or RED in the engine's month-end publication for the date (s3.2). A flag is raised on a customer where any AMBER or RED member is a customer on the credit system, opened by the date.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Cohorts</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>30 September 2022 to 2025. Reached: placed on the watch list, any watch level, within twelve months of the cohort date; groups leaving the book unplaced have not reached it (s4.1, s4.2).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Forecast</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
-        <is>
-          <t>Monitored book at 30 September 2026 only, no new groups (s5.1, s5.2). One probability for flagged groups and one for the rest, from the capture and false-alarm rates (s4.3) with this year's arrival share backed out of the flagged share: the basis whose largest miss is smallest when each closed cohort is predicted from the other three taken together (see Cohorts).</t>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Monitored book at 30 September 2026 only, no new groups (s5.1, s5.2). Each group's chance of reaching the list is the 2022 to 2025 share for groups flagged the same way: flag raised on a customer, flag raised only on a parent or sister company we do not lend to, or not flagged.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Committed exposure</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Facility and obligor extract run at 01:15 on 1 October, after the start-of-day batch; limits taken from the limit history as at 23:00 UTC on 30 September, the end of the day in BST (s1.3, s6.1). Facilities keyed by booking entity and facility number, each counted once in each group with an obligor on it. Non-sterling limits divided by the Group Treasury closing rate (units per pound).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Under £5m; £5m and under £15m; £15m and under £40m; £40m and under £100m; £100m and over (s6.2).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Reference Data quarter-end pack as at 30/09/2026, compiled 08/10/2026.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Credit Risk Monitoring, 27 October 2026.</t>
         </is>

</xml_diff>